<commit_message>
Update 2-22 workbook and download checksums
</commit_message>
<xml_diff>
--- a/2-22 实验八 WPS 表格 公式与函数综合实践-1/step3/分析每月家庭消费明细表.xlsx
+++ b/2-22 实验八 WPS 表格 公式与函数综合实践-1/step3/分析每月家庭消费明细表.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22361" windowHeight="9102"/>
+    <workbookView windowWidth="18468" windowHeight="9420"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -68,11 +68,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="0.00_ "/>
   </numFmts>
   <fonts count="21">
     <font>
@@ -97,12 +98,35 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
       <name val="宋体"/>
@@ -111,7 +135,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FFFA7D00"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -125,6 +149,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF800080"/>
@@ -133,11 +165,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -165,10 +196,10 @@
     </font>
     <font>
       <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -180,9 +211,16 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color rgb="FFFFFFFF"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -190,44 +228,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -248,19 +249,61 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="6" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFCC99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
+        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -272,7 +315,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -284,13 +339,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -302,7 +357,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -314,7 +375,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -326,31 +387,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -362,42 +405,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -410,25 +423,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -543,6 +544,15 @@
       </top>
       <bottom style="medium">
         <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -563,16 +573,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFB2B2B2"/>
+        <color rgb="FF3F3F3F"/>
       </left>
       <right style="thin">
-        <color rgb="FFB2B2B2"/>
+        <color rgb="FF3F3F3F"/>
       </right>
       <top style="thin">
-        <color rgb="FFB2B2B2"/>
+        <color rgb="FF3F3F3F"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -580,8 +590,8 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="medium">
-        <color theme="4"/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -596,16 +606,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color rgb="FFB2B2B2"/>
       </left>
       <right style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color rgb="FFB2B2B2"/>
       </right>
       <top style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color rgb="FFB2B2B2"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -627,15 +637,6 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color theme="4"/>
       </top>
@@ -652,149 +653,149 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="13" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="12" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -811,6 +812,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1151,12 +1155,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:H14"/>
-  <sheetFormatPr defaultColWidth="8.8421052631579" defaultRowHeight="14.1" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="8.84259259259259" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="2" width="8.8421052631579" style="1"/>
-    <col min="3" max="3" width="12.7894736842105" style="1"/>
-    <col min="4" max="4" width="11.6842105263158" style="1"/>
-    <col min="5" max="16380" width="8.8421052631579" style="1"/>
+    <col min="1" max="2" width="8.84259259259259" style="1"/>
+    <col min="3" max="8" width="12.8888888888889" style="1"/>
+    <col min="9" max="16380" width="8.84259259259259" style="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="19" customHeight="1" spans="1:8">
@@ -1192,12 +1195,27 @@
       <c r="B2" s="5">
         <v>1000</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
+      <c r="C2" s="6">
+        <f>B2/21.75+$B$14*8*B2/(21.75*8)</f>
+        <v>183.908045977012</v>
+      </c>
+      <c r="D2" s="6">
+        <f>B2/21.75+$C$14*8*B2/(21.75*8)</f>
+        <v>137.931034482759</v>
+      </c>
+      <c r="E2" s="6">
+        <v>137.931034482759</v>
+      </c>
+      <c r="F2" s="6">
+        <v>137.931034482759</v>
+      </c>
+      <c r="G2" s="6">
+        <v>137.931034482759</v>
+      </c>
+      <c r="H2" s="6">
+        <f>SUM(C2:G2)</f>
+        <v>735.632183908048</v>
+      </c>
     </row>
     <row r="3" ht="19" customHeight="1" spans="1:8">
       <c r="A3" s="4" t="s">
@@ -1206,12 +1224,27 @@
       <c r="B3" s="5">
         <v>1200</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
+      <c r="C3" s="6">
+        <f t="shared" ref="C3:C11" si="0">B3/21.75+$B$14*8*B3/(21.75*8)</f>
+        <v>220.689655172414</v>
+      </c>
+      <c r="D3" s="6">
+        <f t="shared" ref="D3:D11" si="1">B3/21.75+$C$14*8*B3/(21.75*8)</f>
+        <v>165.51724137931</v>
+      </c>
+      <c r="E3" s="6">
+        <v>165.51724137931</v>
+      </c>
+      <c r="F3" s="6">
+        <v>165.51724137931</v>
+      </c>
+      <c r="G3" s="6">
+        <v>165.51724137931</v>
+      </c>
+      <c r="H3" s="6">
+        <f t="shared" ref="H3:H11" si="2">SUM(C3:G3)</f>
+        <v>882.758620689654</v>
+      </c>
     </row>
     <row r="4" ht="19" customHeight="1" spans="1:8">
       <c r="A4" s="4" t="s">
@@ -1220,12 +1253,27 @@
       <c r="B4" s="5">
         <v>1400</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
+      <c r="C4" s="6">
+        <f t="shared" si="0"/>
+        <v>257.471264367816</v>
+      </c>
+      <c r="D4" s="6">
+        <f t="shared" si="1"/>
+        <v>193.103448275862</v>
+      </c>
+      <c r="E4" s="6">
+        <v>193.103448275862</v>
+      </c>
+      <c r="F4" s="6">
+        <v>193.103448275862</v>
+      </c>
+      <c r="G4" s="6">
+        <v>193.103448275862</v>
+      </c>
+      <c r="H4" s="6">
+        <f t="shared" si="2"/>
+        <v>1029.88505747126</v>
+      </c>
     </row>
     <row r="5" ht="19" customHeight="1" spans="1:8">
       <c r="A5" s="4" t="s">
@@ -1234,12 +1282,27 @@
       <c r="B5" s="5">
         <v>1600</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
+      <c r="C5" s="6">
+        <f t="shared" si="0"/>
+        <v>294.252873563218</v>
+      </c>
+      <c r="D5" s="6">
+        <f t="shared" si="1"/>
+        <v>220.689655172414</v>
+      </c>
+      <c r="E5" s="6">
+        <v>220.689655172414</v>
+      </c>
+      <c r="F5" s="6">
+        <v>220.689655172414</v>
+      </c>
+      <c r="G5" s="6">
+        <v>220.689655172414</v>
+      </c>
+      <c r="H5" s="6">
+        <f t="shared" si="2"/>
+        <v>1177.01149425287</v>
+      </c>
     </row>
     <row r="6" ht="19" customHeight="1" spans="1:8">
       <c r="A6" s="4" t="s">
@@ -1248,12 +1311,27 @@
       <c r="B6" s="5">
         <v>1800</v>
       </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
+      <c r="C6" s="6">
+        <f t="shared" si="0"/>
+        <v>331.034482758621</v>
+      </c>
+      <c r="D6" s="6">
+        <f t="shared" si="1"/>
+        <v>248.275862068966</v>
+      </c>
+      <c r="E6" s="6">
+        <v>248.275862068966</v>
+      </c>
+      <c r="F6" s="6">
+        <v>248.275862068966</v>
+      </c>
+      <c r="G6" s="6">
+        <v>248.275862068966</v>
+      </c>
+      <c r="H6" s="6">
+        <f t="shared" si="2"/>
+        <v>1324.13793103449</v>
+      </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:8">
       <c r="A7" s="4" t="s">
@@ -1262,12 +1340,27 @@
       <c r="B7" s="5">
         <v>2000</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
+      <c r="C7" s="6">
+        <f t="shared" si="0"/>
+        <v>367.816091954023</v>
+      </c>
+      <c r="D7" s="6">
+        <f t="shared" si="1"/>
+        <v>275.862068965517</v>
+      </c>
+      <c r="E7" s="6">
+        <v>275.862068965517</v>
+      </c>
+      <c r="F7" s="6">
+        <v>275.862068965517</v>
+      </c>
+      <c r="G7" s="6">
+        <v>275.862068965517</v>
+      </c>
+      <c r="H7" s="6">
+        <f t="shared" si="2"/>
+        <v>1471.26436781609</v>
+      </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:8">
       <c r="A8" s="4" t="s">
@@ -1276,12 +1369,27 @@
       <c r="B8" s="5">
         <v>2200</v>
       </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
+      <c r="C8" s="6">
+        <f t="shared" si="0"/>
+        <v>404.597701149425</v>
+      </c>
+      <c r="D8" s="6">
+        <f t="shared" si="1"/>
+        <v>303.448275862069</v>
+      </c>
+      <c r="E8" s="6">
+        <v>303.448275862069</v>
+      </c>
+      <c r="F8" s="6">
+        <v>303.448275862069</v>
+      </c>
+      <c r="G8" s="6">
+        <v>303.448275862069</v>
+      </c>
+      <c r="H8" s="6">
+        <f t="shared" si="2"/>
+        <v>1618.3908045977</v>
+      </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:8">
       <c r="A9" s="4" t="s">
@@ -1290,12 +1398,27 @@
       <c r="B9" s="5">
         <v>2400</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
+      <c r="C9" s="6">
+        <f t="shared" si="0"/>
+        <v>441.379310344828</v>
+      </c>
+      <c r="D9" s="6">
+        <f t="shared" si="1"/>
+        <v>331.034482758621</v>
+      </c>
+      <c r="E9" s="6">
+        <v>331.034482758621</v>
+      </c>
+      <c r="F9" s="6">
+        <v>331.034482758621</v>
+      </c>
+      <c r="G9" s="6">
+        <v>331.034482758621</v>
+      </c>
+      <c r="H9" s="6">
+        <f t="shared" si="2"/>
+        <v>1765.51724137931</v>
+      </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:8">
       <c r="A10" s="4" t="s">
@@ -1304,12 +1427,27 @@
       <c r="B10" s="5">
         <v>2600</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
+      <c r="C10" s="6">
+        <f t="shared" si="0"/>
+        <v>478.16091954023</v>
+      </c>
+      <c r="D10" s="6">
+        <f t="shared" si="1"/>
+        <v>358.620689655172</v>
+      </c>
+      <c r="E10" s="6">
+        <v>358.620689655172</v>
+      </c>
+      <c r="F10" s="6">
+        <v>358.620689655172</v>
+      </c>
+      <c r="G10" s="6">
+        <v>358.620689655172</v>
+      </c>
+      <c r="H10" s="6">
+        <f t="shared" si="2"/>
+        <v>1912.64367816092</v>
+      </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:8">
       <c r="A11" s="4" t="s">
@@ -1318,33 +1456,48 @@
       <c r="B11" s="5">
         <v>2800</v>
       </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
+      <c r="C11" s="6">
+        <f t="shared" si="0"/>
+        <v>514.942528735632</v>
+      </c>
+      <c r="D11" s="6">
+        <f t="shared" si="1"/>
+        <v>386.206896551724</v>
+      </c>
+      <c r="E11" s="6">
+        <v>386.206896551724</v>
+      </c>
+      <c r="F11" s="6">
+        <v>386.206896551724</v>
+      </c>
+      <c r="G11" s="6">
+        <v>386.206896551724</v>
+      </c>
+      <c r="H11" s="6">
+        <f t="shared" si="2"/>
+        <v>2059.77011494253</v>
+      </c>
     </row>
-    <row r="12" ht="14.85"/>
+    <row r="12" ht="15.15"/>
     <row r="13" spans="1:3">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="7">
+      <c r="B13" s="8">
         <v>44682</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="14" ht="14.85" spans="1:3">
-      <c r="A14" s="9" t="s">
+    <row r="14" ht="15.15" spans="1:3">
+      <c r="A14" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="11">
         <v>3</v>
       </c>
-      <c r="C14" s="11">
+      <c r="C14" s="12">
         <v>2</v>
       </c>
     </row>

</xml_diff>